<commit_message>
@ cleanup: eski "Firmware - yedek" klasoru kaldirildi + PIN_MAPPING.xlsx guncellendi
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
@
</commit_message>
<xml_diff>
--- a/PIN_MAPPING.xlsx
+++ b/PIN_MAPPING.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PressureTransmitter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADBB0A06-9A98-4AF3-9980-342D396A43DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7195672-B23C-4D23-A664-73DD80377630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1605" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Standards Ref" sheetId="3" r:id="rId1"/>
     <sheet name="MCU Pin Map" sheetId="4" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1157,12 +1157,6 @@
     <t>SWD trace, debug only. Diag: see pin 46.</t>
   </si>
   <si>
-    <t>TEST_MODE — production test-mode input (tied/jumper)</t>
-  </si>
-  <si>
-    <t>Test mode. Diag: locked low in safety operation; checked at boot (EN 61508-7 A.18; EN 50402 §6.4.11).</t>
-  </si>
-  <si>
     <t>FLT_TEMP# — temperature fault from B701 TMP108</t>
   </si>
   <si>
@@ -1458,6 +1452,12 @@
   </si>
   <si>
     <t>Note: EN 50402 (electrical apparatus for the detection of combustible/toxic gases — functional safety of fixed gas detection systems) applies to gas detectors only and has been removed from this FMEDA's reference set.</t>
+  </si>
+  <si>
+    <t>TEM_MEAS_ON temperature measurement diode bias. /  TEST_MODE — production test-mode input (tied/jumper)</t>
+  </si>
+  <si>
+    <t>Test mode. Diag: locked low in safety operation; checked at boot (EN 61508-7 A.18; EN 50402 §6.4.11). Measurement on for temp diodes.</t>
   </si>
 </sst>
 </file>
@@ -1729,10 +1729,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2035,7 +2031,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -2052,7 +2048,7 @@
         <v>114</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>115</v>
@@ -2072,7 +2068,7 @@
         <v>119</v>
       </c>
       <c r="E5" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="F5" t="s">
         <v>120</v>
@@ -2092,7 +2088,7 @@
         <v>124</v>
       </c>
       <c r="E6" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="F6" t="s">
         <v>125</v>
@@ -2112,7 +2108,7 @@
         <v>119</v>
       </c>
       <c r="E7" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="F7" t="s">
         <v>129</v>
@@ -2132,7 +2128,7 @@
         <v>124</v>
       </c>
       <c r="E8" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="F8" t="s">
         <v>133</v>
@@ -2152,7 +2148,7 @@
         <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F9" t="s">
         <v>137</v>
@@ -2172,7 +2168,7 @@
         <v>124</v>
       </c>
       <c r="E10" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="F10" t="s">
         <v>141</v>
@@ -2192,7 +2188,7 @@
         <v>119</v>
       </c>
       <c r="E11" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="F11" t="s">
         <v>145</v>
@@ -2212,7 +2208,7 @@
         <v>119</v>
       </c>
       <c r="E12" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="F12" t="s">
         <v>149</v>
@@ -2232,7 +2228,7 @@
         <v>119</v>
       </c>
       <c r="E13" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="F13" t="s">
         <v>153</v>
@@ -2252,7 +2248,7 @@
         <v>124</v>
       </c>
       <c r="E14" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="F14" t="s">
         <v>157</v>
@@ -2272,7 +2268,7 @@
         <v>124</v>
       </c>
       <c r="E15" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="F15" t="s">
         <v>161</v>
@@ -2292,7 +2288,7 @@
         <v>119</v>
       </c>
       <c r="E16" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="F16" t="s">
         <v>165</v>
@@ -2312,7 +2308,7 @@
         <v>169</v>
       </c>
       <c r="E17" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="F17" t="s">
         <v>170</v>
@@ -2365,7 +2361,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -2380,7 +2376,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.3">
@@ -2390,32 +2386,32 @@
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" s="17" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" s="18" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>
@@ -3016,7 +3012,7 @@
         <v>30</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>207</v>
@@ -3025,22 +3021,22 @@
         <v>31</v>
       </c>
       <c r="F20" s="8" t="s">
+        <v>351</v>
+      </c>
+      <c r="G20" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="H20" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="I20" s="16" t="s">
+        <v>352</v>
+      </c>
+      <c r="J20" s="16" t="s">
         <v>353</v>
       </c>
-      <c r="G20" s="16" t="s">
+      <c r="K20" s="9" t="s">
         <v>354</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>354</v>
-      </c>
-      <c r="I20" s="16" t="s">
-        <v>354</v>
-      </c>
-      <c r="J20" s="16" t="s">
-        <v>355</v>
-      </c>
-      <c r="K20" s="9" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3060,22 +3056,22 @@
         <v>209</v>
       </c>
       <c r="F21" s="8" t="s">
+        <v>355</v>
+      </c>
+      <c r="G21" s="16" t="s">
+        <v>356</v>
+      </c>
+      <c r="H21" s="16" t="s">
+        <v>356</v>
+      </c>
+      <c r="I21" s="16" t="s">
+        <v>356</v>
+      </c>
+      <c r="J21" s="16" t="s">
         <v>357</v>
       </c>
-      <c r="G21" s="16" t="s">
+      <c r="K21" s="9" t="s">
         <v>358</v>
-      </c>
-      <c r="H21" s="16" t="s">
-        <v>358</v>
-      </c>
-      <c r="I21" s="16" t="s">
-        <v>358</v>
-      </c>
-      <c r="J21" s="16" t="s">
-        <v>359</v>
-      </c>
-      <c r="K21" s="9" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3165,22 +3161,22 @@
         <v>211</v>
       </c>
       <c r="F24" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>359</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>360</v>
+      </c>
+      <c r="I24" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="J24" s="8" t="s">
         <v>361</v>
       </c>
-      <c r="H24" s="8" t="s">
+      <c r="K24" s="9" t="s">
         <v>362</v>
-      </c>
-      <c r="I24" s="8" t="s">
-        <v>363</v>
-      </c>
-      <c r="J24" s="8" t="s">
-        <v>363</v>
-      </c>
-      <c r="K24" s="9" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3200,22 +3196,22 @@
         <v>213</v>
       </c>
       <c r="F25" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="G25" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="H25" s="16" t="s">
         <v>369</v>
       </c>
-      <c r="G25" s="8" t="s">
+      <c r="I25" s="8" t="s">
         <v>370</v>
       </c>
-      <c r="H25" s="16" t="s">
+      <c r="J25" s="8" t="s">
         <v>371</v>
       </c>
-      <c r="I25" s="8" t="s">
+      <c r="K25" s="9" t="s">
         <v>372</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>373</v>
-      </c>
-      <c r="K25" s="9" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3226,31 +3222,31 @@
         <v>42</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>377</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>378</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="F26" s="16" t="s">
         <v>380</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="G26" s="16" t="s">
+        <v>380</v>
+      </c>
+      <c r="H26" s="8" t="s">
         <v>381</v>
       </c>
-      <c r="F26" s="16" t="s">
+      <c r="I26" s="8" t="s">
         <v>382</v>
       </c>
-      <c r="G26" s="16" t="s">
-        <v>382</v>
-      </c>
-      <c r="H26" s="8" t="s">
+      <c r="J26" s="8" t="s">
         <v>383</v>
       </c>
-      <c r="I26" s="8" t="s">
+      <c r="K26" s="9" t="s">
         <v>384</v>
-      </c>
-      <c r="J26" s="8" t="s">
-        <v>385</v>
-      </c>
-      <c r="K26" s="9" t="s">
-        <v>386</v>
       </c>
     </row>
     <row r="27" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3270,22 +3266,22 @@
         <v>214</v>
       </c>
       <c r="F27" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>374</v>
+      </c>
+      <c r="H27" s="16" t="s">
+        <v>345</v>
+      </c>
+      <c r="I27" s="8" t="s">
         <v>375</v>
       </c>
-      <c r="G27" s="8" t="s">
+      <c r="J27" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="K27" s="9" t="s">
         <v>376</v>
-      </c>
-      <c r="H27" s="16" t="s">
-        <v>347</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>377</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>377</v>
-      </c>
-      <c r="K27" s="9" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3410,22 +3406,22 @@
         <v>204</v>
       </c>
       <c r="F31" s="8" t="s">
+        <v>363</v>
+      </c>
+      <c r="G31" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="H31" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="I31" s="16" t="s">
+        <v>364</v>
+      </c>
+      <c r="J31" s="16" t="s">
         <v>365</v>
       </c>
-      <c r="G31" s="16" t="s">
+      <c r="K31" s="9" t="s">
         <v>366</v>
-      </c>
-      <c r="H31" s="16" t="s">
-        <v>366</v>
-      </c>
-      <c r="I31" s="16" t="s">
-        <v>366</v>
-      </c>
-      <c r="J31" s="16" t="s">
-        <v>367</v>
-      </c>
-      <c r="K31" s="9" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3439,28 +3435,28 @@
         <v>54</v>
       </c>
       <c r="D32" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="F32" s="16" t="s">
         <v>387</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="G32" s="16" t="s">
+        <v>387</v>
+      </c>
+      <c r="H32" s="16" t="s">
         <v>388</v>
       </c>
-      <c r="F32" s="16" t="s">
+      <c r="I32" s="8" t="s">
         <v>389</v>
       </c>
-      <c r="G32" s="16" t="s">
-        <v>389</v>
-      </c>
-      <c r="H32" s="16" t="s">
+      <c r="J32" s="8" t="s">
         <v>390</v>
       </c>
-      <c r="I32" s="8" t="s">
+      <c r="K32" s="9" t="s">
         <v>391</v>
-      </c>
-      <c r="J32" s="8" t="s">
-        <v>392</v>
-      </c>
-      <c r="K32" s="9" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="33" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3471,7 +3467,7 @@
         <v>55</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>203</v>
@@ -3480,22 +3476,22 @@
         <v>204</v>
       </c>
       <c r="F33" s="16" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="H33" s="16" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="I33" s="16" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="J33" s="16" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="34" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3655,10 +3651,10 @@
         <v>218</v>
       </c>
       <c r="F38" s="16" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="G38" s="16" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="H38" s="7" t="s">
         <v>301</v>
@@ -3667,10 +3663,10 @@
         <v>301</v>
       </c>
       <c r="J38" s="16" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="39" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3690,10 +3686,10 @@
         <v>220</v>
       </c>
       <c r="F39" s="16" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="H39" s="7" t="s">
         <v>302</v>
@@ -3702,10 +3698,10 @@
         <v>302</v>
       </c>
       <c r="J39" s="16" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="K39" s="9" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3725,10 +3721,10 @@
         <v>222</v>
       </c>
       <c r="F40" s="16" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="G40" s="16" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="H40" s="7" t="s">
         <v>303</v>
@@ -3737,10 +3733,10 @@
         <v>303</v>
       </c>
       <c r="J40" s="16" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="K40" s="9" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
     </row>
     <row r="41" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3760,10 +3756,10 @@
         <v>204</v>
       </c>
       <c r="F41" s="16" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="H41" s="7" t="s">
         <v>304</v>
@@ -3772,10 +3768,10 @@
         <v>304</v>
       </c>
       <c r="J41" s="16" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="K41" s="9" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="42" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3795,10 +3791,10 @@
         <v>204</v>
       </c>
       <c r="F42" s="16" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="G42" s="16" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>305</v>
@@ -3807,10 +3803,10 @@
         <v>305</v>
       </c>
       <c r="J42" s="16" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="K42" s="9" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="43" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3830,10 +3826,10 @@
         <v>204</v>
       </c>
       <c r="F43" s="16" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="H43" s="7" t="s">
         <v>306</v>
@@ -3842,10 +3838,10 @@
         <v>306</v>
       </c>
       <c r="J43" s="16" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="K43" s="9" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3865,10 +3861,10 @@
         <v>227</v>
       </c>
       <c r="F44" s="16" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="H44" s="7" t="s">
         <v>307</v>
@@ -3877,10 +3873,10 @@
         <v>307</v>
       </c>
       <c r="J44" s="16" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="K44" s="9" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="45" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3900,10 +3896,10 @@
         <v>229</v>
       </c>
       <c r="F45" s="16" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="H45" s="7" t="s">
         <v>308</v>
@@ -3912,10 +3908,10 @@
         <v>308</v>
       </c>
       <c r="J45" s="16" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="K45" s="9" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -3970,16 +3966,16 @@
         <v>204</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="I47" s="7" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="J47" s="8" t="s">
         <v>291</v>
@@ -4355,22 +4351,22 @@
         <v>204</v>
       </c>
       <c r="F58" s="8" t="s">
+        <v>346</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="I58" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="J58" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="G58" s="7" t="s">
+      <c r="K58" s="9" t="s">
         <v>349</v>
-      </c>
-      <c r="H58" s="7" t="s">
-        <v>349</v>
-      </c>
-      <c r="I58" s="7" t="s">
-        <v>349</v>
-      </c>
-      <c r="J58" s="8" t="s">
-        <v>350</v>
-      </c>
-      <c r="K58" s="9" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4425,22 +4421,22 @@
         <v>204</v>
       </c>
       <c r="F60" s="7" t="s">
-        <v>333</v>
+        <v>432</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>333</v>
+        <v>432</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>333</v>
+        <v>432</v>
       </c>
       <c r="I60" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="J60" s="8" t="s">
-        <v>333</v>
+        <v>432</v>
+      </c>
+      <c r="J60" s="7" t="s">
+        <v>432</v>
       </c>
       <c r="K60" s="9" t="s">
-        <v>334</v>
+        <v>433</v>
       </c>
     </row>
     <row r="61" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4460,22 +4456,22 @@
         <v>241</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="I61" s="7" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J61" s="8" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="K61" s="9" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
     </row>
     <row r="62" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4495,22 +4491,22 @@
         <v>204</v>
       </c>
       <c r="F62" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="H62" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="I62" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J62" s="8" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="K62" s="9" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4530,22 +4526,22 @@
         <v>242</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="G63" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="I63" s="7" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J63" s="8" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="K63" s="9" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="64" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4565,22 +4561,22 @@
         <v>245</v>
       </c>
       <c r="F64" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="G64" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="H64" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="I64" s="7" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="J64" s="8" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="K64" s="9" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4600,22 +4596,22 @@
         <v>247</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="I65" s="7" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J65" s="8" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="K65" s="9" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="66" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -4635,22 +4631,22 @@
         <v>248</v>
       </c>
       <c r="F66" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="H66" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="I66" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J66" s="8" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="K66" s="9" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="67" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>